<commit_message>
feat(attendance): update date format to dd/MM/yyyy without seconds, add DateInput component, and remove sample download button
</commit_message>
<xml_diff>
--- a/samples/ZKTeco_LX50_Asistencia_Ejemplo.xlsx
+++ b/samples/ZKTeco_LX50_Asistencia_Ejemplo.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="43">
   <si>
     <t>Reporte de Asistencia - Terminal Biométrica ZKTeco LX50</t>
   </si>
   <si>
-    <t>Periodo: 2026-09-01 ~ 2026-09-30 | Terminal: LX50_RH_PRINCIPAL</t>
+    <t>Periodo: 01/09/2026 ~ 30/09/2026 | Terminal: LX50_RH_PRINCIPAL</t>
   </si>
   <si>
     <t>No. AC</t>
@@ -47,7 +47,7 @@
     <t>Carlos Mendoza Flores</t>
   </si>
   <si>
-    <t>2026-09-15 07:58:22</t>
+    <t>15/09/2026 07:58</t>
   </si>
   <si>
     <t>Entrada</t>
@@ -65,19 +65,19 @@
     <t>LX50</t>
   </si>
   <si>
-    <t>2026-09-15 14:02:45</t>
+    <t>15/09/2026 14:02</t>
   </si>
   <si>
     <t>Salida Almuerzo</t>
   </si>
   <si>
-    <t>2026-09-15 15:01:10</t>
+    <t>15/09/2026 15:01</t>
   </si>
   <si>
     <t>Regreso Almuerzo</t>
   </si>
   <si>
-    <t>2026-09-15 18:05:30</t>
+    <t>15/09/2026 18:05</t>
   </si>
   <si>
     <t>Salida</t>
@@ -86,58 +86,55 @@
     <t>Mariana Ruiz Galindo</t>
   </si>
   <si>
-    <t>2026-09-15 08:04:12</t>
-  </si>
-  <si>
-    <t>2026-09-15 17:30:44</t>
+    <t>15/09/2026 08:04</t>
+  </si>
+  <si>
+    <t>15/09/2026 17:30</t>
   </si>
   <si>
     <t>Jorge Luis Hernandez</t>
   </si>
   <si>
-    <t>2026-09-15 08:15:03</t>
+    <t>15/09/2026 08:15</t>
   </si>
   <si>
     <t>Contraseña</t>
   </si>
   <si>
-    <t>2026-09-15 18:00:19</t>
+    <t>15/09/2026 18:00</t>
   </si>
   <si>
     <t>Laura Patricia Ortiz</t>
   </si>
   <si>
-    <t>2026-09-15 08:00:00</t>
+    <t>15/09/2026 08:00</t>
   </si>
   <si>
     <t>Tarjeta</t>
   </si>
   <si>
-    <t>2026-09-15 18:10:55</t>
-  </si>
-  <si>
-    <t>2026-09-15 08:02:11</t>
-  </si>
-  <si>
-    <t>2026-09-15 17:59:33</t>
+    <t>15/09/2026 18:10</t>
+  </si>
+  <si>
+    <t>15/09/2026 08:02</t>
+  </si>
+  <si>
+    <t>15/09/2026 17:59</t>
   </si>
   <si>
     <t>Roberto Sanchez Peña</t>
   </si>
   <si>
-    <t>2026-09-15 07:55:10</t>
-  </si>
-  <si>
-    <t>2026-09-15 07:55:25</t>
-  </si>
-  <si>
-    <t>2026-09-15 17:02:11</t>
+    <t>15/09/2026 07:55</t>
+  </si>
+  <si>
+    <t>15/09/2026 17:02</t>
   </si>
   <si>
     <t>Empleado Fantasma</t>
   </si>
   <si>
-    <t>2026-09-15 08:30:00</t>
+    <t>15/09/2026 08:30</t>
   </si>
   <si>
     <t>Beatriz Domínguez</t>
@@ -216,9 +213,9 @@
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="54.84375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="55.4765625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="19.12109375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="17.640625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="15.4296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="15.53515625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="12.265625" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="9.125" customWidth="true" bestFit="true"/>
@@ -609,7 +606,7 @@
         <v>36</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D18" t="s" s="0">
         <v>12</v>
@@ -635,7 +632,7 @@
         <v>36</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s" s="0">
         <v>22</v>
@@ -658,10 +655,10 @@
         <v>14</v>
       </c>
       <c r="B20" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C20" t="s" s="0">
         <v>40</v>
-      </c>
-      <c r="C20" t="s" s="0">
-        <v>41</v>
       </c>
       <c r="D20" t="s" s="0">
         <v>12</v>
@@ -684,10 +681,10 @@
         <v>107.0</v>
       </c>
       <c r="B21" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s" s="0">
         <v>42</v>
-      </c>
-      <c r="C21" t="s" s="0">
-        <v>43</v>
       </c>
       <c r="D21" t="s" s="0">
         <v>12</v>

</xml_diff>